<commit_message>
Add themes page and refresh ORCiD list
Update _data/MVLS LTS ORCiD.xlsx from the Form export: 66 -> 70 members.
The weekly job reads this file from the repo, so the four members who
joined since 25 June had not been picked up.

Add automatic theme grouping for the SoTL outputs:

- R/fetch_abstracts.R pulls abstracts and subject terms from OpenAlex,
  falling back to Crossref, cached in _data/abstracts.json and only
  topped up on later runs.
- R/classify_themes.R scores each output against seven topic themes plus
  a cross-cutting methods tag, weighting title over journal over
  abstract. Multi-label, capped at three themes per output.
- _data/theme_overrides.csv applies manual corrections last.
- themes.qmd renders the grouping, with the ten most recent outputs per
  theme and a filterable table of everything.

Themes were revised after the August 2026 symposium. The grouping is a
browsing aid, not a structure the network has adopted.
</commit_message>
<xml_diff>
--- a/_data/MVLS LTS ORCiD.xlsx
+++ b/_data/MVLS LTS ORCiD.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30413"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gla-my.sharepoint.com/personal/emily_nordmann_glasgow_ac_uk/Documents/04_Leadership-and-Governance/mvls-lts/_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A388971-5ACC-410D-85FD-39C1563EE96A}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7197BECC-1FC6-4ED4-8413-47E3E98CD32B}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="170">
   <si>
     <t>Id</t>
   </si>
@@ -508,13 +508,52 @@
   </si>
   <si>
     <t>https://orcid.org/0000-0001-8771-4185</t>
+  </si>
+  <si>
+    <t>Jenny.Clancy@glasgow.ac.uk</t>
+  </si>
+  <si>
+    <t>Jenny Clancy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0002-1568-2046 </t>
+  </si>
+  <si>
+    <t>Jennifer.Hammond@glasgow.ac.uk</t>
+  </si>
+  <si>
+    <t>Jennifer Hammond</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0009-0002-1963-2545</t>
+  </si>
+  <si>
+    <t>Courtney.TaylorBrowneLuka@glasgow.ac.uk</t>
+  </si>
+  <si>
+    <t>Courtney Taylor Browne Luka</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0002-2819-0673</t>
+  </si>
+  <si>
+    <t>Sandy.Wilson@glasgow.ac.uk</t>
+  </si>
+  <si>
+    <t>Sandy Wilson</t>
+  </si>
+  <si>
+    <t>Graduate School</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0002-9313-4280</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -593,8 +632,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:G68" totalsRowShown="0">
-  <autoFilter ref="A1:G68" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:G72" totalsRowShown="0">
+  <autoFilter ref="A1:G72" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id" dataDxfId="4">
       <extLst>
@@ -649,7 +688,7 @@
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{839C7E11-91E4-4DBD-9C5D-0DEA604FA9AC}">
-      <xlmsforms:msForm id="KVxybjp2UE-B8i4lTwEzyKAHhjrab3lLkx60RR1iKjNUOTVNTEMwVE02SEhMQ0ZZODExQktLVThBSiQlQCNjPTEu" isFormConnected="1" maxResponseId="4" latestEventMarker="3">
+      <xlmsforms:msForm id="KVxybjp2UE-B8i4lTwEzyKAHhjrab3lLkx60RR1iKjNUOTVNTEMwVE02SEhMQ0ZZODExQktLVThBSiQlQCNjPTEu" isFormConnected="1" maxResponseId="8" latestEventMarker="7">
         <xlmsforms:syncedQuestionId>id</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>startDate</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>submitDate</xlmsforms:syncedQuestionId>
@@ -960,13 +999,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G68"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:G72"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="7" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -989,7 +1028,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1012,7 +1051,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7">
       <c r="D3" s="1"/>
       <c r="E3" s="1" t="s">
         <v>11</v>
@@ -1024,7 +1063,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7">
       <c r="D4" s="1"/>
       <c r="E4" s="1" t="s">
         <v>14</v>
@@ -1036,7 +1075,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7">
       <c r="D5" s="1"/>
       <c r="E5" s="1" t="s">
         <v>16</v>
@@ -1048,7 +1087,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7">
       <c r="D6" s="1"/>
       <c r="E6" s="1" t="s">
         <v>18</v>
@@ -1060,7 +1099,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7">
       <c r="D7" s="1"/>
       <c r="E7" s="1" t="s">
         <v>21</v>
@@ -1072,7 +1111,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7">
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="s">
         <v>23</v>
@@ -1084,7 +1123,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7">
       <c r="D9" s="1"/>
       <c r="E9" s="1" t="s">
         <v>25</v>
@@ -1096,7 +1135,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7">
       <c r="D10" s="1"/>
       <c r="E10" s="1" t="s">
         <v>27</v>
@@ -1108,7 +1147,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7">
       <c r="D11" s="1"/>
       <c r="E11" s="1" t="s">
         <v>30</v>
@@ -1120,7 +1159,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7">
       <c r="D12" s="1"/>
       <c r="E12" s="1" t="s">
         <v>32</v>
@@ -1132,7 +1171,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7">
       <c r="D13" s="1"/>
       <c r="E13" s="1" t="s">
         <v>35</v>
@@ -1144,7 +1183,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7">
       <c r="D14" s="1"/>
       <c r="E14" s="1" t="s">
         <v>38</v>
@@ -1156,7 +1195,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7">
       <c r="D15" s="1"/>
       <c r="E15" s="1" t="s">
         <v>40</v>
@@ -1168,7 +1207,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7">
       <c r="D16" s="1"/>
       <c r="E16" s="1" t="s">
         <v>42</v>
@@ -1180,7 +1219,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="4:7">
       <c r="D17" s="1"/>
       <c r="E17" s="1" t="s">
         <v>44</v>
@@ -1192,7 +1231,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="4:7">
       <c r="D18" s="1"/>
       <c r="E18" s="1" t="s">
         <v>46</v>
@@ -1204,7 +1243,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="19" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="4:7">
       <c r="D19" s="1"/>
       <c r="E19" s="1" t="s">
         <v>48</v>
@@ -1216,7 +1255,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="20" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="4:7">
       <c r="D20" s="1"/>
       <c r="E20" s="1" t="s">
         <v>50</v>
@@ -1228,7 +1267,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="4:7">
       <c r="D21" s="1"/>
       <c r="E21" s="1" t="s">
         <v>52</v>
@@ -1240,7 +1279,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="4:7">
       <c r="D22" s="1"/>
       <c r="E22" s="1" t="s">
         <v>55</v>
@@ -1252,7 +1291,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="4:7">
       <c r="D23" s="1"/>
       <c r="E23" s="1" t="s">
         <v>57</v>
@@ -1264,7 +1303,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="24" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="4:7">
       <c r="D24" s="1"/>
       <c r="E24" s="1" t="s">
         <v>59</v>
@@ -1276,7 +1315,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="4:7">
       <c r="D25" s="1"/>
       <c r="E25" s="1" t="s">
         <v>61</v>
@@ -1288,7 +1327,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="26" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="4:7">
       <c r="D26" s="1"/>
       <c r="E26" s="1" t="s">
         <v>64</v>
@@ -1300,7 +1339,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="4:7">
       <c r="D27" s="1"/>
       <c r="E27" s="1" t="s">
         <v>66</v>
@@ -1312,7 +1351,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="28" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="4:7">
       <c r="D28" s="1"/>
       <c r="E28" s="1" t="s">
         <v>69</v>
@@ -1324,7 +1363,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="29" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="4:7">
       <c r="D29" s="1"/>
       <c r="E29" s="1" t="s">
         <v>71</v>
@@ -1336,7 +1375,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="4:7">
       <c r="D30" s="1"/>
       <c r="E30" s="1" t="s">
         <v>73</v>
@@ -1348,7 +1387,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="31" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="4:7">
       <c r="D31" s="1"/>
       <c r="E31" s="1" t="s">
         <v>75</v>
@@ -1360,7 +1399,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="32" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="4:7">
       <c r="D32" s="1"/>
       <c r="E32" s="1" t="s">
         <v>77</v>
@@ -1372,7 +1411,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="33" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="4:7">
       <c r="D33" s="1"/>
       <c r="E33" s="1" t="s">
         <v>79</v>
@@ -1384,7 +1423,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="34" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="4:7">
       <c r="D34" s="1"/>
       <c r="E34" s="1" t="s">
         <v>82</v>
@@ -1396,7 +1435,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="35" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="4:7">
       <c r="D35" s="1"/>
       <c r="E35" s="1" t="s">
         <v>84</v>
@@ -1408,7 +1447,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="36" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="4:7">
       <c r="D36" s="1"/>
       <c r="E36" s="1" t="s">
         <v>86</v>
@@ -1420,7 +1459,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="37" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="4:7">
       <c r="D37" s="1"/>
       <c r="E37" s="1" t="s">
         <v>88</v>
@@ -1432,7 +1471,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="38" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="4:7">
       <c r="D38" s="1"/>
       <c r="E38" s="1" t="s">
         <v>90</v>
@@ -1444,7 +1483,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="39" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="4:7">
       <c r="D39" s="1"/>
       <c r="E39" s="1" t="s">
         <v>92</v>
@@ -1456,7 +1495,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="40" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="4:7">
       <c r="D40" s="1"/>
       <c r="E40" s="1" t="s">
         <v>94</v>
@@ -1468,7 +1507,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="41" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="4:7">
       <c r="D41" s="1"/>
       <c r="E41" s="1" t="s">
         <v>96</v>
@@ -1480,7 +1519,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="42" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="4:7">
       <c r="D42" s="1"/>
       <c r="E42" s="1" t="s">
         <v>98</v>
@@ -1492,7 +1531,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="43" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="4:7">
       <c r="D43" s="1"/>
       <c r="E43" s="1" t="s">
         <v>100</v>
@@ -1504,7 +1543,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="44" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="4:7">
       <c r="D44" s="1"/>
       <c r="E44" s="1" t="s">
         <v>102</v>
@@ -1516,7 +1555,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="45" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="4:7">
       <c r="D45" s="1"/>
       <c r="E45" s="1" t="s">
         <v>104</v>
@@ -1528,7 +1567,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="46" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="4:7">
       <c r="D46" s="1"/>
       <c r="E46" s="1" t="s">
         <v>106</v>
@@ -1540,7 +1579,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="47" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="47" spans="4:7">
       <c r="D47" s="1"/>
       <c r="E47" s="1" t="s">
         <v>108</v>
@@ -1552,7 +1591,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="48" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="4:7">
       <c r="D48" s="1"/>
       <c r="E48" s="1" t="s">
         <v>110</v>
@@ -1564,7 +1603,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="49" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="4:7">
       <c r="D49" s="1"/>
       <c r="E49" s="1" t="s">
         <v>112</v>
@@ -1576,7 +1615,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="50" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="4:7">
       <c r="D50" s="1"/>
       <c r="E50" s="1" t="s">
         <v>114</v>
@@ -1588,7 +1627,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="51" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="4:7">
       <c r="D51" s="1"/>
       <c r="E51" s="1" t="s">
         <v>116</v>
@@ -1600,7 +1639,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="52" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="4:7">
       <c r="D52" s="1"/>
       <c r="E52" s="1" t="s">
         <v>119</v>
@@ -1612,7 +1651,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="53" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="4:7">
       <c r="D53" s="1"/>
       <c r="E53" s="1" t="s">
         <v>121</v>
@@ -1624,7 +1663,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="54" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="4:7">
       <c r="D54" s="1"/>
       <c r="E54" s="1" t="s">
         <v>123</v>
@@ -1636,7 +1675,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="55" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="4:7">
       <c r="D55" s="1"/>
       <c r="E55" s="1" t="s">
         <v>125</v>
@@ -1648,7 +1687,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="56" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="4:7">
       <c r="D56" s="1"/>
       <c r="E56" s="1" t="s">
         <v>127</v>
@@ -1660,7 +1699,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="57" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="4:7">
       <c r="D57" s="1"/>
       <c r="E57" s="1" t="s">
         <v>129</v>
@@ -1672,7 +1711,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="58" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="4:7">
       <c r="D58" s="1"/>
       <c r="E58" s="1" t="s">
         <v>131</v>
@@ -1684,7 +1723,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="59" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="4:7">
       <c r="D59" s="1"/>
       <c r="E59" s="1" t="s">
         <v>132</v>
@@ -1696,7 +1735,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="60" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="4:7">
       <c r="D60" s="1"/>
       <c r="E60" s="1" t="s">
         <v>134</v>
@@ -1708,7 +1747,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="61" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="4:7">
       <c r="D61" s="1"/>
       <c r="E61" s="1" t="s">
         <v>137</v>
@@ -1720,7 +1759,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="62" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="4:7">
       <c r="D62" s="1"/>
       <c r="E62" s="1" t="s">
         <v>139</v>
@@ -1732,7 +1771,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="63" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="4:7">
       <c r="D63" s="1"/>
       <c r="E63" s="1" t="s">
         <v>141</v>
@@ -1744,7 +1783,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="64" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="4:7">
       <c r="D64" s="1"/>
       <c r="E64" s="1" t="s">
         <v>143</v>
@@ -1756,7 +1795,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7">
       <c r="D65" s="1"/>
       <c r="E65" s="1" t="s">
         <v>145</v>
@@ -1768,7 +1807,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7">
       <c r="D66" s="1"/>
       <c r="E66" s="1" t="s">
         <v>147</v>
@@ -1780,7 +1819,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7">
       <c r="A67">
         <v>3</v>
       </c>
@@ -1803,8 +1842,8 @@
         <v>152</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A68" s="4">
+    <row r="68" spans="1:7">
+      <c r="A68">
         <v>4</v>
       </c>
       <c r="B68">
@@ -1824,6 +1863,98 @@
       </c>
       <c r="G68" s="3" t="s">
         <v>156</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="15">
+      <c r="A69" s="4">
+        <v>5</v>
+      </c>
+      <c r="B69">
+        <v>46217.6531944444</v>
+      </c>
+      <c r="C69">
+        <v>46217.6546296296</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" ht="15">
+      <c r="A70" s="4">
+        <v>6</v>
+      </c>
+      <c r="B70">
+        <v>46217.742696759298</v>
+      </c>
+      <c r="C70">
+        <v>46217.743993055599</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" ht="15">
+      <c r="A71" s="4">
+        <v>7</v>
+      </c>
+      <c r="B71">
+        <v>46253.4205671296</v>
+      </c>
+      <c r="C71">
+        <v>46253.422476851803</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" ht="15">
+      <c r="A72" s="4">
+        <v>8</v>
+      </c>
+      <c r="B72">
+        <v>46254.5945601852</v>
+      </c>
+      <c r="C72">
+        <v>46254.595439814802</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="G72" s="3" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>

</xml_diff>